<commit_message>
feat：filter displaying habits in calendar
</commit_message>
<xml_diff>
--- a/移动应用开发大作业评分表.xlsx
+++ b/移动应用开发大作业评分表.xlsx
@@ -1886,7 +1886,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="15">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:4">
@@ -1934,7 +1934,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" ht="51" customHeight="1" spans="1:4">
@@ -1967,7 +1967,9 @@
       <c r="C18" s="14">
         <v>3</v>
       </c>
-      <c r="D18" s="15"/>
+      <c r="D18" s="15">
+        <v>3</v>
+      </c>
     </row>
     <row r="19" ht="51" customHeight="1" spans="1:4">
       <c r="A19" s="28"/>
@@ -1989,7 +1991,9 @@
       <c r="C20" s="14">
         <v>4</v>
       </c>
-      <c r="D20" s="15"/>
+      <c r="D20" s="15">
+        <v>4</v>
+      </c>
     </row>
     <row r="21" ht="51" customHeight="1" spans="1:4">
       <c r="A21" s="26"/>
@@ -2059,7 +2063,9 @@
       <c r="C26" s="34">
         <v>2</v>
       </c>
-      <c r="D26" s="34"/>
+      <c r="D26" s="34">
+        <v>2</v>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:4">
       <c r="A27" s="26"/>
@@ -2248,7 +2254,7 @@
       </c>
       <c r="D48" s="46">
         <f>SUM(D8:D47)</f>
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>